<commit_message>
venv and pd folder rename
</commit_message>
<xml_diff>
--- a/outputs/1 N NO 1_ch00_measurements.xlsx
+++ b/outputs/1 N NO 1_ch00_measurements.xlsx
@@ -241,7 +241,7 @@
       <row>2</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="23260050" cy="8020050"/>
+    <ext cx="23231475" cy="8010525"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -301,7 +301,7 @@
       <row>2</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7143750" cy="8420100"/>
+    <ext cx="7143750" cy="8401050"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -2140,7 +2140,7 @@
         <v>127.9221818181818</v>
       </c>
       <c r="D6" t="n">
-        <v>35.73035463249191</v>
+        <v>35.73035463249192</v>
       </c>
       <c r="E6" t="n">
         <v>79.941</v>
@@ -2233,7 +2233,7 @@
         <v>28.68318181818181</v>
       </c>
       <c r="D9" t="n">
-        <v>5.500083632421997</v>
+        <v>5.500083632421998</v>
       </c>
       <c r="E9" t="n">
         <v>20.99</v>
@@ -2388,7 +2388,7 @@
         <v>150.5916363636364</v>
       </c>
       <c r="D14" t="n">
-        <v>17.85421527971883</v>
+        <v>17.85421527971884</v>
       </c>
       <c r="E14" t="n">
         <v>129.98</v>

</xml_diff>